<commit_message>
#8 Ribbon Added In BOM
</commit_message>
<xml_diff>
--- a/Design-Files/SecondaryPCB-airbnb/BOM/eSpark_BOM_SecondaryPCB-airbnb.xlsx
+++ b/Design-Files/SecondaryPCB-airbnb/BOM/eSpark_BOM_SecondaryPCB-airbnb.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="5 Boards" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="145">
   <si>
     <t>Component list</t>
   </si>
@@ -422,6 +422,39 @@
   </si>
   <si>
     <t>Unit Cost (10 Boards)</t>
+  </si>
+  <si>
+    <t>Peripheral</t>
+  </si>
+  <si>
+    <t>FFCE2008T108000-300</t>
+  </si>
+  <si>
+    <t>0.3mm~0.3mm 20 0.5mm Same Side 8cm P=0.5mm FFC/FPC Connect Cables ROHS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cvilux </t>
+  </si>
+  <si>
+    <t>C918683</t>
+  </si>
+  <si>
+    <t>JS05A-20P-050-4-8</t>
+  </si>
+  <si>
+    <t>0.3mm~0.3mm 20 0.5mm Same Side 5cm P=0.5mm FFC/FPC Connect Cables ROHS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ribbon Cable 80mm </t>
+  </si>
+  <si>
+    <t>Ribbon Cable 50mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JUSHUO </t>
+  </si>
+  <si>
+    <t>C2857502</t>
   </si>
 </sst>
 </file>
@@ -1054,6 +1087,56 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="23" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1065,18 +1148,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1086,54 +1157,16 @@
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="23" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1532,7 +1565,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:S27"/>
+  <dimension ref="A1:S29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="26" customWidth="1"/>
@@ -1566,15 +1599,15 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="60"/>
-      <c r="N1" s="60"/>
-      <c r="O1" s="60"/>
-      <c r="P1" s="60"/>
-      <c r="Q1" s="60"/>
-      <c r="R1" s="60"/>
-      <c r="S1" s="61"/>
+      <c r="K1" s="78"/>
+      <c r="L1" s="78"/>
+      <c r="M1" s="78"/>
+      <c r="N1" s="78"/>
+      <c r="O1" s="78"/>
+      <c r="P1" s="78"/>
+      <c r="Q1" s="78"/>
+      <c r="R1" s="78"/>
+      <c r="S1" s="79"/>
     </row>
     <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1624,7 +1657,7 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
-      <c r="S3" s="62"/>
+      <c r="S3" s="80"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1649,7 +1682,7 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="63"/>
+      <c r="S4" s="81"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1674,7 +1707,7 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="6"/>
-      <c r="S5" s="63"/>
+      <c r="S5" s="81"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1695,7 +1728,7 @@
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
-      <c r="S6" s="63"/>
+      <c r="S6" s="81"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1716,7 +1749,7 @@
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
-      <c r="S7" s="63"/>
+      <c r="S7" s="81"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1737,7 +1770,7 @@
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="63"/>
+      <c r="S8" s="81"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -1839,7 +1872,7 @@
       <c r="N10" s="37">
         <v>100</v>
       </c>
-      <c r="O10" s="82" t="s">
+      <c r="O10" s="72" t="s">
         <v>126</v>
       </c>
       <c r="P10" s="38">
@@ -1854,451 +1887,451 @@
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
-      <c r="B11" s="71">
+      <c r="B11" s="61">
         <f t="shared" ref="B11:B24" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
-      <c r="C11" s="72" t="s">
+      <c r="C11" s="62" t="s">
         <v>9</v>
       </c>
-      <c r="D11" s="73" t="s">
+      <c r="D11" s="63" t="s">
         <v>21</v>
       </c>
-      <c r="E11" s="73" t="s">
+      <c r="E11" s="63" t="s">
         <v>36</v>
       </c>
-      <c r="F11" s="73" t="s">
+      <c r="F11" s="63" t="s">
         <v>52</v>
       </c>
-      <c r="G11" s="73" t="s">
+      <c r="G11" s="63" t="s">
         <v>65</v>
       </c>
-      <c r="H11" s="73" t="s">
+      <c r="H11" s="63" t="s">
         <v>78</v>
       </c>
-      <c r="I11" s="73" t="s">
-        <v>127</v>
-      </c>
-      <c r="J11" s="73" t="s">
+      <c r="I11" s="63" t="s">
+        <v>127</v>
+      </c>
+      <c r="J11" s="63" t="s">
         <v>90</v>
       </c>
-      <c r="K11" s="73" t="s">
+      <c r="K11" s="63" t="s">
         <v>104</v>
       </c>
-      <c r="L11" s="73">
+      <c r="L11" s="63">
         <v>1</v>
       </c>
-      <c r="M11" s="73">
+      <c r="M11" s="63">
         <f t="shared" ref="M11" si="1">L11*5</f>
         <v>5</v>
       </c>
-      <c r="N11" s="73">
+      <c r="N11" s="63">
         <v>20</v>
       </c>
-      <c r="O11" s="84" t="s">
+      <c r="O11" s="74" t="s">
         <v>126</v>
       </c>
-      <c r="P11" s="74">
+      <c r="P11" s="64">
         <v>2.3300000000000001E-2</v>
       </c>
-      <c r="Q11" s="74">
+      <c r="Q11" s="64">
         <f t="shared" ref="Q11" si="2">P11*N11</f>
         <v>0.46600000000000003</v>
       </c>
-      <c r="R11" s="73"/>
-      <c r="S11" s="73"/>
+      <c r="R11" s="63"/>
+      <c r="S11" s="63"/>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
-      <c r="B12" s="77">
+      <c r="B12" s="67">
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
-      <c r="C12" s="72" t="s">
+      <c r="C12" s="62" t="s">
         <v>9</v>
       </c>
-      <c r="D12" s="79" t="s">
+      <c r="D12" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="79" t="s">
+      <c r="E12" s="69" t="s">
         <v>37</v>
       </c>
-      <c r="F12" s="79" t="s">
+      <c r="F12" s="69" t="s">
         <v>53</v>
       </c>
-      <c r="G12" s="79" t="s">
+      <c r="G12" s="69" t="s">
         <v>66</v>
       </c>
-      <c r="H12" s="79" t="s">
+      <c r="H12" s="69" t="s">
         <v>77</v>
       </c>
-      <c r="I12" s="79" t="s">
-        <v>127</v>
-      </c>
-      <c r="J12" s="79" t="s">
+      <c r="I12" s="69" t="s">
+        <v>127</v>
+      </c>
+      <c r="J12" s="69" t="s">
         <v>91</v>
       </c>
-      <c r="K12" s="79" t="s">
+      <c r="K12" s="69" t="s">
         <v>105</v>
       </c>
-      <c r="L12" s="79">
+      <c r="L12" s="69">
         <v>2</v>
       </c>
-      <c r="M12" s="79">
+      <c r="M12" s="69">
         <f>L12*5</f>
         <v>10</v>
       </c>
       <c r="N12" s="37">
         <v>20</v>
       </c>
-      <c r="O12" s="82" t="s">
+      <c r="O12" s="72" t="s">
         <v>126</v>
       </c>
       <c r="P12" s="38">
         <v>3.5200000000000002E-2</v>
       </c>
-      <c r="Q12" s="80">
+      <c r="Q12" s="70">
         <f>P12*N12</f>
         <v>0.70400000000000007</v>
       </c>
-      <c r="R12" s="79"/>
-      <c r="S12" s="75"/>
+      <c r="R12" s="69"/>
+      <c r="S12" s="65"/>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
-      <c r="B13" s="77">
+      <c r="B13" s="67">
         <f>ROW(B13) - ROW($B$9)</f>
         <v>4</v>
       </c>
-      <c r="C13" s="72" t="s">
+      <c r="C13" s="62" t="s">
         <v>9</v>
       </c>
-      <c r="D13" s="79" t="s">
+      <c r="D13" s="69" t="s">
         <v>23</v>
       </c>
-      <c r="E13" s="79" t="s">
+      <c r="E13" s="69" t="s">
         <v>38</v>
       </c>
-      <c r="F13" s="79" t="s">
+      <c r="F13" s="69" t="s">
         <v>52</v>
       </c>
-      <c r="G13" s="79" t="s">
+      <c r="G13" s="69" t="s">
         <v>67</v>
       </c>
-      <c r="H13" s="79" t="s">
+      <c r="H13" s="69" t="s">
         <v>79</v>
       </c>
-      <c r="I13" s="79" t="s">
-        <v>127</v>
-      </c>
-      <c r="J13" s="79" t="s">
+      <c r="I13" s="69" t="s">
+        <v>127</v>
+      </c>
+      <c r="J13" s="69" t="s">
         <v>92</v>
       </c>
-      <c r="K13" s="79" t="s">
+      <c r="K13" s="69" t="s">
         <v>107</v>
       </c>
-      <c r="L13" s="79">
+      <c r="L13" s="69">
         <v>4</v>
       </c>
-      <c r="M13" s="79">
+      <c r="M13" s="69">
         <f>L13*5</f>
         <v>20</v>
       </c>
-      <c r="N13" s="79">
+      <c r="N13" s="69">
         <v>50</v>
       </c>
-      <c r="O13" s="83" t="s">
+      <c r="O13" s="73" t="s">
         <v>126</v>
       </c>
-      <c r="P13" s="80">
+      <c r="P13" s="70">
         <v>1.0800000000000001E-2</v>
       </c>
-      <c r="Q13" s="80">
+      <c r="Q13" s="70">
         <f>P13*N13</f>
         <v>0.54</v>
       </c>
-      <c r="R13" s="79"/>
-      <c r="S13" s="75"/>
+      <c r="R13" s="69"/>
+      <c r="S13" s="65"/>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
-      <c r="B14" s="71">
+      <c r="B14" s="61">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="72" t="s">
+      <c r="C14" s="62" t="s">
         <v>9</v>
       </c>
-      <c r="D14" s="73" t="s">
+      <c r="D14" s="63" t="s">
         <v>24</v>
       </c>
-      <c r="E14" s="73" t="s">
+      <c r="E14" s="63" t="s">
         <v>39</v>
       </c>
-      <c r="F14" s="73" t="s">
+      <c r="F14" s="63" t="s">
         <v>52</v>
       </c>
-      <c r="G14" s="73" t="s">
+      <c r="G14" s="63" t="s">
         <v>68</v>
       </c>
-      <c r="H14" s="73" t="s">
+      <c r="H14" s="63" t="s">
         <v>77</v>
       </c>
-      <c r="I14" s="73" t="s">
-        <v>127</v>
-      </c>
-      <c r="J14" s="73" t="s">
+      <c r="I14" s="63" t="s">
+        <v>127</v>
+      </c>
+      <c r="J14" s="63" t="s">
         <v>93</v>
       </c>
-      <c r="K14" s="73" t="s">
+      <c r="K14" s="63" t="s">
         <v>108</v>
       </c>
-      <c r="L14" s="73">
+      <c r="L14" s="63">
         <v>1</v>
       </c>
-      <c r="M14" s="73">
+      <c r="M14" s="63">
         <f t="shared" ref="M14:M15" si="3">L14*5</f>
         <v>5</v>
       </c>
-      <c r="N14" s="73">
+      <c r="N14" s="63">
         <v>100</v>
       </c>
-      <c r="O14" s="84" t="s">
+      <c r="O14" s="74" t="s">
         <v>126</v>
       </c>
-      <c r="P14" s="74">
+      <c r="P14" s="64">
         <v>1.1000000000000001E-3</v>
       </c>
-      <c r="Q14" s="74">
+      <c r="Q14" s="64">
         <f t="shared" ref="Q14:Q15" si="4">P14*N14</f>
         <v>0.11</v>
       </c>
-      <c r="R14" s="73"/>
-      <c r="S14" s="75"/>
+      <c r="R14" s="63"/>
+      <c r="S14" s="65"/>
     </row>
     <row r="15" spans="1:19" ht="24" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
-      <c r="B15" s="71">
+      <c r="B15" s="61">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="72" t="s">
+      <c r="C15" s="62" t="s">
         <v>9</v>
       </c>
       <c r="D15" s="49" t="s">
         <v>128</v>
       </c>
-      <c r="E15" s="73" t="s">
+      <c r="E15" s="63" t="s">
         <v>40</v>
       </c>
-      <c r="F15" s="73" t="s">
+      <c r="F15" s="63" t="s">
         <v>52</v>
       </c>
-      <c r="G15" s="73" t="s">
+      <c r="G15" s="63" t="s">
         <v>69</v>
       </c>
-      <c r="H15" s="73" t="s">
+      <c r="H15" s="63" t="s">
         <v>77</v>
       </c>
-      <c r="I15" s="73" t="s">
-        <v>127</v>
-      </c>
-      <c r="J15" s="73" t="s">
+      <c r="I15" s="63" t="s">
+        <v>127</v>
+      </c>
+      <c r="J15" s="63" t="s">
         <v>94</v>
       </c>
-      <c r="K15" s="73" t="s">
+      <c r="K15" s="63" t="s">
         <v>106</v>
       </c>
-      <c r="L15" s="73">
+      <c r="L15" s="63">
         <v>11</v>
       </c>
-      <c r="M15" s="73">
+      <c r="M15" s="63">
         <f t="shared" si="3"/>
         <v>55</v>
       </c>
       <c r="N15" s="37">
         <v>100</v>
       </c>
-      <c r="O15" s="82" t="s">
+      <c r="O15" s="72" t="s">
         <v>126</v>
       </c>
       <c r="P15" s="38">
         <v>1.1000000000000001E-3</v>
       </c>
-      <c r="Q15" s="74">
+      <c r="Q15" s="64">
         <f t="shared" si="4"/>
         <v>0.11</v>
       </c>
-      <c r="R15" s="73"/>
-      <c r="S15" s="75"/>
+      <c r="R15" s="63"/>
+      <c r="S15" s="65"/>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
-      <c r="B16" s="77">
+      <c r="B16" s="67">
         <f>ROW(B16) - ROW($B$9)</f>
         <v>7</v>
       </c>
-      <c r="C16" s="78" t="s">
+      <c r="C16" s="68" t="s">
         <v>10</v>
       </c>
-      <c r="D16" s="79" t="s">
+      <c r="D16" s="69" t="s">
         <v>25</v>
       </c>
-      <c r="E16" s="79" t="s">
+      <c r="E16" s="69" t="s">
         <v>41</v>
       </c>
-      <c r="F16" s="79" t="s">
+      <c r="F16" s="69" t="s">
         <v>54</v>
       </c>
-      <c r="G16" s="79" t="s">
+      <c r="G16" s="69" t="s">
         <v>70</v>
       </c>
-      <c r="H16" s="79" t="s">
+      <c r="H16" s="69" t="s">
         <v>80</v>
       </c>
-      <c r="I16" s="79" t="s">
-        <v>127</v>
-      </c>
-      <c r="J16" s="79" t="s">
+      <c r="I16" s="69" t="s">
+        <v>127</v>
+      </c>
+      <c r="J16" s="69" t="s">
         <v>95</v>
       </c>
-      <c r="K16" s="79" t="s">
+      <c r="K16" s="69" t="s">
         <v>109</v>
       </c>
-      <c r="L16" s="79">
+      <c r="L16" s="69">
         <v>7</v>
       </c>
-      <c r="M16" s="79">
+      <c r="M16" s="69">
         <f>L16*5</f>
         <v>35</v>
       </c>
       <c r="N16" s="37">
         <v>100</v>
       </c>
-      <c r="O16" s="82" t="s">
+      <c r="O16" s="72" t="s">
         <v>126</v>
       </c>
       <c r="P16" s="38">
         <v>5.5999999999999999E-3</v>
       </c>
-      <c r="Q16" s="80">
+      <c r="Q16" s="70">
         <f>P16*N16</f>
         <v>0.55999999999999994</v>
       </c>
-      <c r="R16" s="79"/>
-      <c r="S16" s="75"/>
+      <c r="R16" s="69"/>
+      <c r="S16" s="65"/>
     </row>
     <row r="17" spans="1:19" ht="36" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
-      <c r="B17" s="71">
+      <c r="B17" s="61">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="72" t="s">
+      <c r="C17" s="62" t="s">
         <v>11</v>
       </c>
-      <c r="D17" s="73" t="s">
+      <c r="D17" s="63" t="s">
         <v>26</v>
       </c>
       <c r="E17" s="49" t="s">
         <v>42</v>
       </c>
-      <c r="F17" s="73" t="s">
+      <c r="F17" s="63" t="s">
         <v>125</v>
       </c>
-      <c r="G17" s="73" t="s">
+      <c r="G17" s="63" t="s">
         <v>55</v>
       </c>
-      <c r="H17" s="73" t="s">
+      <c r="H17" s="63" t="s">
         <v>81</v>
       </c>
-      <c r="I17" s="73" t="s">
-        <v>127</v>
-      </c>
-      <c r="J17" s="73" t="s">
+      <c r="I17" s="63" t="s">
+        <v>127</v>
+      </c>
+      <c r="J17" s="63" t="s">
         <v>96</v>
       </c>
-      <c r="K17" s="73" t="s">
-        <v>127</v>
-      </c>
-      <c r="L17" s="73">
+      <c r="K17" s="63" t="s">
+        <v>127</v>
+      </c>
+      <c r="L17" s="63">
         <v>1</v>
       </c>
-      <c r="M17" s="73">
+      <c r="M17" s="63">
         <f t="shared" ref="M17" si="5">L17*5</f>
         <v>5</v>
       </c>
       <c r="N17" s="49">
         <v>10</v>
       </c>
-      <c r="O17" s="82" t="s">
+      <c r="O17" s="72" t="s">
         <v>126</v>
       </c>
       <c r="P17" s="50">
         <v>8.6599999999999996E-2</v>
       </c>
-      <c r="Q17" s="74">
+      <c r="Q17" s="64">
         <f t="shared" ref="Q17" si="6">P17*N17</f>
         <v>0.86599999999999999</v>
       </c>
-      <c r="R17" s="73"/>
-      <c r="S17" s="75"/>
+      <c r="R17" s="63"/>
+      <c r="S17" s="65"/>
     </row>
     <row r="18" spans="1:19" ht="24" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
-      <c r="B18" s="77">
+      <c r="B18" s="67">
         <f>ROW(B18) - ROW($B$9)</f>
         <v>9</v>
       </c>
-      <c r="C18" s="78" t="s">
+      <c r="C18" s="68" t="s">
         <v>12</v>
       </c>
-      <c r="D18" s="79" t="s">
+      <c r="D18" s="69" t="s">
         <v>27</v>
       </c>
       <c r="E18" s="37" t="s">
         <v>43</v>
       </c>
-      <c r="F18" s="79" t="s">
+      <c r="F18" s="69" t="s">
         <v>125</v>
       </c>
-      <c r="G18" s="79" t="s">
+      <c r="G18" s="69" t="s">
         <v>56</v>
       </c>
-      <c r="H18" s="79" t="s">
+      <c r="H18" s="69" t="s">
         <v>82</v>
       </c>
-      <c r="I18" s="79" t="s">
-        <v>127</v>
-      </c>
-      <c r="J18" s="79" t="s">
+      <c r="I18" s="69" t="s">
+        <v>127</v>
+      </c>
+      <c r="J18" s="69" t="s">
         <v>97</v>
       </c>
-      <c r="K18" s="79" t="s">
-        <v>127</v>
-      </c>
-      <c r="L18" s="79">
+      <c r="K18" s="69" t="s">
+        <v>127</v>
+      </c>
+      <c r="L18" s="69">
         <v>5</v>
       </c>
-      <c r="M18" s="79">
+      <c r="M18" s="69">
         <f>L18*5</f>
         <v>25</v>
       </c>
-      <c r="N18" s="79">
+      <c r="N18" s="69">
         <v>30</v>
       </c>
-      <c r="O18" s="83" t="s">
+      <c r="O18" s="73" t="s">
         <v>126</v>
       </c>
-      <c r="P18" s="80">
+      <c r="P18" s="70">
         <v>0.2044</v>
       </c>
-      <c r="Q18" s="80">
+      <c r="Q18" s="70">
         <f>P18*N18</f>
         <v>6.1319999999999997</v>
       </c>
-      <c r="R18" s="79"/>
-      <c r="S18" s="75"/>
+      <c r="R18" s="69"/>
+      <c r="S18" s="65"/>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
@@ -2309,437 +2342,549 @@
       <c r="C19" s="51" t="s">
         <v>13</v>
       </c>
-      <c r="D19" s="85" t="s">
+      <c r="D19" s="75" t="s">
         <v>28</v>
       </c>
-      <c r="E19" s="85" t="s">
+      <c r="E19" s="75" t="s">
         <v>44</v>
       </c>
-      <c r="F19" s="85" t="s">
-        <v>127</v>
-      </c>
-      <c r="G19" s="85" t="s">
+      <c r="F19" s="75" t="s">
+        <v>127</v>
+      </c>
+      <c r="G19" s="75" t="s">
         <v>57</v>
       </c>
-      <c r="H19" s="85" t="s">
-        <v>127</v>
-      </c>
-      <c r="I19" s="85" t="s">
-        <v>127</v>
-      </c>
-      <c r="J19" s="85" t="s">
-        <v>127</v>
-      </c>
-      <c r="K19" s="85" t="s">
-        <v>127</v>
-      </c>
-      <c r="L19" s="85">
+      <c r="H19" s="75" t="s">
+        <v>127</v>
+      </c>
+      <c r="I19" s="75" t="s">
+        <v>127</v>
+      </c>
+      <c r="J19" s="75" t="s">
+        <v>127</v>
+      </c>
+      <c r="K19" s="75" t="s">
+        <v>127</v>
+      </c>
+      <c r="L19" s="75">
         <v>1</v>
       </c>
-      <c r="M19" s="85">
+      <c r="M19" s="75">
         <f t="shared" ref="M19:M20" si="7">L19*5</f>
         <v>5</v>
       </c>
-      <c r="N19" s="85" t="s">
-        <v>127</v>
-      </c>
-      <c r="O19" s="85" t="s">
-        <v>127</v>
-      </c>
-      <c r="P19" s="86" t="s">
-        <v>127</v>
-      </c>
-      <c r="Q19" s="86" t="s">
-        <v>127</v>
-      </c>
-      <c r="R19" s="85"/>
-      <c r="S19" s="87"/>
+      <c r="N19" s="75" t="s">
+        <v>127</v>
+      </c>
+      <c r="O19" s="75" t="s">
+        <v>127</v>
+      </c>
+      <c r="P19" s="76" t="s">
+        <v>127</v>
+      </c>
+      <c r="Q19" s="76" t="s">
+        <v>127</v>
+      </c>
+      <c r="R19" s="75"/>
+      <c r="S19" s="77"/>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
-      <c r="B20" s="71">
+      <c r="B20" s="61">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C20" s="72" t="s">
+      <c r="C20" s="62" t="s">
         <v>14</v>
       </c>
-      <c r="D20" s="73" t="s">
+      <c r="D20" s="63" t="s">
         <v>29</v>
       </c>
-      <c r="E20" s="73" t="s">
+      <c r="E20" s="63" t="s">
         <v>45</v>
       </c>
-      <c r="F20" s="73" t="s">
+      <c r="F20" s="63" t="s">
         <v>58</v>
       </c>
-      <c r="G20" s="73" t="s">
+      <c r="G20" s="63" t="s">
         <v>71</v>
       </c>
-      <c r="H20" s="73" t="s">
+      <c r="H20" s="63" t="s">
         <v>83</v>
       </c>
-      <c r="I20" s="73"/>
-      <c r="J20" s="73" t="s">
+      <c r="I20" s="63"/>
+      <c r="J20" s="63" t="s">
         <v>98</v>
       </c>
-      <c r="K20" s="73" t="s">
+      <c r="K20" s="63" t="s">
         <v>111</v>
       </c>
-      <c r="L20" s="73">
+      <c r="L20" s="63">
         <v>1</v>
       </c>
-      <c r="M20" s="73">
+      <c r="M20" s="63">
         <f t="shared" si="7"/>
         <v>5</v>
       </c>
-      <c r="N20" s="73">
+      <c r="N20" s="63">
         <v>50</v>
       </c>
-      <c r="O20" s="84" t="s">
+      <c r="O20" s="74" t="s">
         <v>126</v>
       </c>
-      <c r="P20" s="74">
+      <c r="P20" s="64">
         <v>3.5999999999999999E-3</v>
       </c>
-      <c r="Q20" s="74">
+      <c r="Q20" s="64">
         <f t="shared" ref="Q20" si="8">P20*N20</f>
         <v>0.18</v>
       </c>
-      <c r="R20" s="73"/>
-      <c r="S20" s="75"/>
+      <c r="R20" s="63"/>
+      <c r="S20" s="65"/>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
-      <c r="B21" s="77">
+      <c r="B21" s="67">
         <f>ROW(B21) - ROW($B$9)</f>
         <v>12</v>
       </c>
-      <c r="C21" s="78" t="s">
+      <c r="C21" s="68" t="s">
         <v>14</v>
       </c>
-      <c r="D21" s="79" t="s">
+      <c r="D21" s="69" t="s">
         <v>129</v>
       </c>
-      <c r="E21" s="79" t="s">
+      <c r="E21" s="69" t="s">
         <v>46</v>
       </c>
-      <c r="F21" s="79" t="s">
+      <c r="F21" s="69" t="s">
         <v>59</v>
       </c>
-      <c r="G21" s="79" t="s">
+      <c r="G21" s="69" t="s">
         <v>72</v>
       </c>
-      <c r="H21" s="79" t="s">
+      <c r="H21" s="69" t="s">
         <v>77</v>
       </c>
-      <c r="I21" s="79" t="s">
-        <v>127</v>
-      </c>
-      <c r="J21" s="79" t="s">
+      <c r="I21" s="69" t="s">
+        <v>127</v>
+      </c>
+      <c r="J21" s="69" t="s">
         <v>99</v>
       </c>
-      <c r="K21" s="79" t="s">
+      <c r="K21" s="69" t="s">
         <v>110</v>
       </c>
-      <c r="L21" s="79">
-        <v>4</v>
-      </c>
-      <c r="M21" s="79">
+      <c r="L21" s="69">
+        <v>5</v>
+      </c>
+      <c r="M21" s="69">
         <f>L21*5</f>
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="N21" s="49">
         <v>100</v>
       </c>
-      <c r="O21" s="82" t="s">
+      <c r="O21" s="72" t="s">
         <v>126</v>
       </c>
       <c r="P21" s="50">
         <v>1E-3</v>
       </c>
-      <c r="Q21" s="80">
+      <c r="Q21" s="70">
         <f>P21*N21</f>
         <v>0.1</v>
       </c>
-      <c r="R21" s="79"/>
-      <c r="S21" s="75"/>
+      <c r="R21" s="69"/>
+      <c r="S21" s="65"/>
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
-      <c r="B22" s="71">
+      <c r="B22" s="61">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C22" s="72" t="s">
+      <c r="C22" s="62" t="s">
         <v>15</v>
       </c>
-      <c r="D22" s="73" t="s">
+      <c r="D22" s="63" t="s">
         <v>30</v>
       </c>
-      <c r="E22" s="73" t="s">
+      <c r="E22" s="63" t="s">
         <v>47</v>
       </c>
-      <c r="F22" s="73" t="s">
+      <c r="F22" s="63" t="s">
         <v>60</v>
       </c>
-      <c r="G22" s="73" t="s">
+      <c r="G22" s="63" t="s">
         <v>73</v>
       </c>
-      <c r="H22" s="73" t="s">
+      <c r="H22" s="63" t="s">
         <v>84</v>
       </c>
-      <c r="I22" s="73" t="s">
-        <v>127</v>
-      </c>
-      <c r="J22" s="73"/>
-      <c r="K22" s="73" t="s">
-        <v>127</v>
-      </c>
-      <c r="L22" s="73">
+      <c r="I22" s="63" t="s">
+        <v>127</v>
+      </c>
+      <c r="J22" s="63"/>
+      <c r="K22" s="63" t="s">
+        <v>127</v>
+      </c>
+      <c r="L22" s="63">
         <v>1</v>
       </c>
-      <c r="M22" s="73">
+      <c r="M22" s="63">
         <f t="shared" ref="M22" si="9">L22*5</f>
         <v>5</v>
       </c>
-      <c r="N22" s="73"/>
-      <c r="O22" s="73"/>
-      <c r="P22" s="74"/>
-      <c r="Q22" s="74">
+      <c r="N22" s="63"/>
+      <c r="O22" s="63"/>
+      <c r="P22" s="64"/>
+      <c r="Q22" s="64">
         <f t="shared" ref="Q22" si="10">P22*N22</f>
         <v>0</v>
       </c>
-      <c r="R22" s="73"/>
-      <c r="S22" s="75"/>
+      <c r="R22" s="63"/>
+      <c r="S22" s="65"/>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
-      <c r="B23" s="77">
+      <c r="B23" s="67">
         <f>ROW(B23) - ROW($B$9)</f>
         <v>14</v>
       </c>
-      <c r="C23" s="78" t="s">
+      <c r="C23" s="68" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="79" t="s">
+      <c r="D23" s="69" t="s">
         <v>31</v>
       </c>
-      <c r="E23" s="79" t="s">
+      <c r="E23" s="69" t="s">
         <v>48</v>
       </c>
-      <c r="F23" s="79" t="s">
+      <c r="F23" s="69" t="s">
         <v>61</v>
       </c>
-      <c r="G23" s="79" t="s">
+      <c r="G23" s="69" t="s">
         <v>74</v>
       </c>
-      <c r="H23" s="79" t="s">
+      <c r="H23" s="69" t="s">
         <v>85</v>
       </c>
-      <c r="I23" s="79" t="s">
-        <v>127</v>
-      </c>
-      <c r="J23" s="79" t="s">
+      <c r="I23" s="69" t="s">
+        <v>127</v>
+      </c>
+      <c r="J23" s="69" t="s">
         <v>100</v>
       </c>
-      <c r="K23" s="79" t="s">
-        <v>127</v>
-      </c>
-      <c r="L23" s="79">
+      <c r="K23" s="69" t="s">
+        <v>127</v>
+      </c>
+      <c r="L23" s="69">
         <v>1</v>
       </c>
-      <c r="M23" s="79">
+      <c r="M23" s="69">
         <f>L23*5</f>
         <v>5</v>
       </c>
-      <c r="N23" s="79">
+      <c r="N23" s="69">
         <v>6</v>
       </c>
-      <c r="O23" s="83" t="s">
+      <c r="O23" s="73" t="s">
         <v>126</v>
       </c>
-      <c r="P23" s="80">
+      <c r="P23" s="70">
         <v>0.3866</v>
       </c>
-      <c r="Q23" s="80">
+      <c r="Q23" s="70">
         <f>P23*N23</f>
         <v>2.3195999999999999</v>
       </c>
-      <c r="R23" s="79"/>
-      <c r="S23" s="75"/>
+      <c r="R23" s="69"/>
+      <c r="S23" s="65"/>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
-      <c r="B24" s="71">
+      <c r="B24" s="61">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C24" s="72" t="s">
+      <c r="C24" s="62" t="s">
         <v>17</v>
       </c>
-      <c r="D24" s="73" t="s">
+      <c r="D24" s="63" t="s">
         <v>32</v>
       </c>
-      <c r="E24" s="73" t="s">
+      <c r="E24" s="63" t="s">
         <v>49</v>
       </c>
-      <c r="F24" s="73" t="s">
+      <c r="F24" s="63" t="s">
         <v>125</v>
       </c>
-      <c r="G24" s="73" t="s">
+      <c r="G24" s="63" t="s">
         <v>62</v>
       </c>
-      <c r="H24" s="73" t="s">
+      <c r="H24" s="63" t="s">
         <v>86</v>
       </c>
-      <c r="I24" s="73" t="s">
-        <v>127</v>
-      </c>
-      <c r="J24" s="73" t="s">
+      <c r="I24" s="63" t="s">
+        <v>127</v>
+      </c>
+      <c r="J24" s="63" t="s">
         <v>101</v>
       </c>
-      <c r="K24" s="73" t="s">
-        <v>127</v>
-      </c>
-      <c r="L24" s="73">
+      <c r="K24" s="63" t="s">
+        <v>127</v>
+      </c>
+      <c r="L24" s="63">
         <v>4</v>
       </c>
-      <c r="M24" s="73">
+      <c r="M24" s="63">
         <f t="shared" ref="M24" si="11">L24*5</f>
         <v>20</v>
       </c>
-      <c r="N24" s="73">
+      <c r="N24" s="63">
         <v>21</v>
       </c>
-      <c r="O24" s="84" t="s">
+      <c r="O24" s="74" t="s">
         <v>126</v>
       </c>
-      <c r="P24" s="74">
+      <c r="P24" s="64">
         <v>1.9424999999999999</v>
       </c>
-      <c r="Q24" s="74">
+      <c r="Q24" s="64">
         <f t="shared" ref="Q24" si="12">P24*N24</f>
         <v>40.792499999999997</v>
       </c>
-      <c r="R24" s="73"/>
-      <c r="S24" s="75"/>
+      <c r="R24" s="63"/>
+      <c r="S24" s="65"/>
     </row>
     <row r="25" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
-      <c r="B25" s="77">
+      <c r="B25" s="67">
         <f>ROW(B25) - ROW($B$9)</f>
         <v>16</v>
       </c>
-      <c r="C25" s="78" t="s">
+      <c r="C25" s="68" t="s">
         <v>18</v>
       </c>
-      <c r="D25" s="79" t="s">
+      <c r="D25" s="69" t="s">
         <v>33</v>
       </c>
-      <c r="E25" s="79" t="s">
+      <c r="E25" s="69" t="s">
         <v>50</v>
       </c>
-      <c r="F25" s="79" t="s">
+      <c r="F25" s="69" t="s">
         <v>125</v>
       </c>
-      <c r="G25" s="79" t="s">
+      <c r="G25" s="69" t="s">
         <v>75</v>
       </c>
-      <c r="H25" s="79" t="s">
+      <c r="H25" s="69" t="s">
         <v>87</v>
       </c>
-      <c r="I25" s="79" t="s">
-        <v>127</v>
-      </c>
-      <c r="J25" s="79" t="s">
+      <c r="I25" s="69" t="s">
+        <v>127</v>
+      </c>
+      <c r="J25" s="69" t="s">
         <v>102</v>
       </c>
-      <c r="K25" s="79" t="s">
+      <c r="K25" s="69" t="s">
         <v>112</v>
       </c>
-      <c r="L25" s="79">
+      <c r="L25" s="69">
         <v>1</v>
       </c>
-      <c r="M25" s="79">
+      <c r="M25" s="69">
         <f>L25*5</f>
         <v>5</v>
       </c>
-      <c r="N25" s="79">
+      <c r="N25" s="69">
         <v>6</v>
       </c>
-      <c r="O25" s="83" t="s">
+      <c r="O25" s="73" t="s">
         <v>126</v>
       </c>
-      <c r="P25" s="80">
+      <c r="P25" s="70">
         <v>0.86070000000000002</v>
       </c>
-      <c r="Q25" s="80">
+      <c r="Q25" s="70">
         <f>P25*N25</f>
         <v>5.1642000000000001</v>
       </c>
-      <c r="R25" s="79"/>
-      <c r="S25" s="81"/>
-    </row>
-    <row r="26" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R25" s="69"/>
+      <c r="S25" s="71"/>
+    </row>
+    <row r="26" spans="1:19" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
-      <c r="B26" s="39"/>
-      <c r="C26" s="40"/>
-      <c r="D26" s="41"/>
-      <c r="E26" s="42"/>
-      <c r="F26" s="43"/>
-      <c r="G26" s="44"/>
-      <c r="H26" s="43"/>
-      <c r="I26" s="44"/>
-      <c r="J26" s="43"/>
-      <c r="K26" s="44"/>
-      <c r="L26" s="44"/>
-      <c r="M26" s="44"/>
-      <c r="N26" s="68" t="s">
+      <c r="B26" s="67">
+        <f t="shared" ref="B26:B27" si="13">ROW(B26) - ROW($B$9)</f>
+        <v>17</v>
+      </c>
+      <c r="C26" s="68" t="s">
+        <v>134</v>
+      </c>
+      <c r="D26" s="69" t="s">
+        <v>141</v>
+      </c>
+      <c r="E26" s="37" t="s">
+        <v>136</v>
+      </c>
+      <c r="F26" s="69" t="s">
+        <v>127</v>
+      </c>
+      <c r="G26" s="37" t="s">
+        <v>135</v>
+      </c>
+      <c r="H26" s="69" t="s">
+        <v>137</v>
+      </c>
+      <c r="I26" s="63" t="s">
+        <v>127</v>
+      </c>
+      <c r="J26" s="69" t="s">
+        <v>138</v>
+      </c>
+      <c r="K26" s="69" t="s">
+        <v>127</v>
+      </c>
+      <c r="L26" s="69">
+        <v>1</v>
+      </c>
+      <c r="M26" s="69">
+        <f>L26*5</f>
         <v>5</v>
       </c>
-      <c r="O26" s="69"/>
-      <c r="P26" s="69"/>
-      <c r="Q26" s="47">
-        <f>SUM(Q10:Q25)</f>
-        <v>58.284299999999995</v>
-      </c>
-      <c r="R26" s="64"/>
-      <c r="S26" s="65"/>
-    </row>
-    <row r="27" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="N26" s="69">
+        <v>6</v>
+      </c>
+      <c r="O26" s="73" t="s">
+        <v>126</v>
+      </c>
+      <c r="P26" s="70">
+        <v>0.17219999999999999</v>
+      </c>
+      <c r="Q26" s="70">
+        <f>P26*N26</f>
+        <v>1.0331999999999999</v>
+      </c>
+      <c r="R26" s="69"/>
+      <c r="S26" s="71"/>
+    </row>
+    <row r="27" spans="1:19" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
-      <c r="B27" s="25"/>
-      <c r="C27" s="36"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="10"/>
-      <c r="F27" s="10"/>
-      <c r="G27" s="10"/>
-      <c r="H27" s="10"/>
-      <c r="I27" s="10"/>
-      <c r="J27" s="10"/>
-      <c r="K27" s="10"/>
-      <c r="L27" s="10"/>
-      <c r="M27" s="10"/>
-      <c r="N27" s="68" t="s">
+      <c r="B27" s="67">
+        <f t="shared" si="13"/>
+        <v>18</v>
+      </c>
+      <c r="C27" s="68" t="s">
+        <v>134</v>
+      </c>
+      <c r="D27" s="69" t="s">
+        <v>142</v>
+      </c>
+      <c r="E27" s="37" t="s">
+        <v>140</v>
+      </c>
+      <c r="F27" s="69" t="s">
+        <v>127</v>
+      </c>
+      <c r="G27" s="69" t="s">
+        <v>139</v>
+      </c>
+      <c r="H27" s="69" t="s">
+        <v>143</v>
+      </c>
+      <c r="I27" s="69" t="s">
+        <v>127</v>
+      </c>
+      <c r="J27" s="69" t="s">
+        <v>144</v>
+      </c>
+      <c r="K27" s="69" t="s">
+        <v>127</v>
+      </c>
+      <c r="L27" s="69">
+        <v>1</v>
+      </c>
+      <c r="M27" s="69">
+        <f>L27*5</f>
+        <v>5</v>
+      </c>
+      <c r="N27" s="69">
+        <v>10</v>
+      </c>
+      <c r="O27" s="73" t="s">
+        <v>126</v>
+      </c>
+      <c r="P27" s="70">
+        <v>8.0600000000000005E-2</v>
+      </c>
+      <c r="Q27" s="70">
+        <f>P27*N27</f>
+        <v>0.80600000000000005</v>
+      </c>
+      <c r="R27" s="69"/>
+      <c r="S27" s="71"/>
+    </row>
+    <row r="28" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="1"/>
+      <c r="B28" s="39"/>
+      <c r="C28" s="40"/>
+      <c r="D28" s="41"/>
+      <c r="E28" s="42"/>
+      <c r="F28" s="43"/>
+      <c r="G28" s="44"/>
+      <c r="H28" s="43"/>
+      <c r="I28" s="44"/>
+      <c r="J28" s="43"/>
+      <c r="K28" s="44"/>
+      <c r="L28" s="44"/>
+      <c r="M28" s="44"/>
+      <c r="N28" s="82" t="s">
+        <v>5</v>
+      </c>
+      <c r="O28" s="83"/>
+      <c r="P28" s="83"/>
+      <c r="Q28" s="47">
+        <f>SUM(Q10:Q27)</f>
+        <v>60.123499999999993</v>
+      </c>
+      <c r="R28" s="84"/>
+      <c r="S28" s="85"/>
+    </row>
+    <row r="29" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="1"/>
+      <c r="B29" s="25"/>
+      <c r="C29" s="36"/>
+      <c r="D29" s="9"/>
+      <c r="E29" s="10"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="10"/>
+      <c r="H29" s="10"/>
+      <c r="I29" s="10"/>
+      <c r="J29" s="10"/>
+      <c r="K29" s="10"/>
+      <c r="L29" s="10"/>
+      <c r="M29" s="10"/>
+      <c r="N29" s="82" t="s">
         <v>6</v>
       </c>
-      <c r="O27" s="69"/>
-      <c r="P27" s="69"/>
-      <c r="Q27" s="48">
-        <f>Q26/5</f>
-        <v>11.656859999999998</v>
-      </c>
-      <c r="R27" s="66"/>
-      <c r="S27" s="67"/>
+      <c r="O29" s="83"/>
+      <c r="P29" s="83"/>
+      <c r="Q29" s="48">
+        <f>Q28/5</f>
+        <v>12.024699999999999</v>
+      </c>
+      <c r="R29" s="86"/>
+      <c r="S29" s="87"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="K1:S1"/>
     <mergeCell ref="S3:S8"/>
-    <mergeCell ref="N26:P26"/>
-    <mergeCell ref="R26:S27"/>
-    <mergeCell ref="N27:P27"/>
+    <mergeCell ref="N28:P28"/>
+    <mergeCell ref="R28:S29"/>
+    <mergeCell ref="N29:P29"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="O10" r:id="rId1"/>
@@ -2756,16 +2901,18 @@
     <hyperlink ref="O13" r:id="rId12"/>
     <hyperlink ref="O14" r:id="rId13"/>
     <hyperlink ref="O20" r:id="rId14"/>
+    <hyperlink ref="O26" r:id="rId15"/>
+    <hyperlink ref="O27" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId15"/>
-  <drawing r:id="rId16"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId17"/>
+  <drawing r:id="rId18"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S27"/>
+  <dimension ref="A1:S29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
@@ -2799,15 +2946,15 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="60"/>
-      <c r="N1" s="60"/>
-      <c r="O1" s="60"/>
-      <c r="P1" s="60"/>
-      <c r="Q1" s="60"/>
-      <c r="R1" s="60"/>
-      <c r="S1" s="61"/>
+      <c r="K1" s="78"/>
+      <c r="L1" s="78"/>
+      <c r="M1" s="78"/>
+      <c r="N1" s="78"/>
+      <c r="O1" s="78"/>
+      <c r="P1" s="78"/>
+      <c r="Q1" s="78"/>
+      <c r="R1" s="78"/>
+      <c r="S1" s="79"/>
     </row>
     <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2857,7 +3004,7 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
-      <c r="S3" s="62"/>
+      <c r="S3" s="80"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -2882,7 +3029,7 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="63"/>
+      <c r="S4" s="81"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -2907,7 +3054,7 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="6"/>
-      <c r="S5" s="63"/>
+      <c r="S5" s="81"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -2928,7 +3075,7 @@
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
-      <c r="S6" s="63"/>
+      <c r="S6" s="81"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -2949,7 +3096,7 @@
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
-      <c r="S7" s="63"/>
+      <c r="S7" s="81"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -2970,7 +3117,7 @@
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="63"/>
+      <c r="S8" s="81"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -3072,7 +3219,7 @@
       <c r="N10" s="37">
         <v>200</v>
       </c>
-      <c r="O10" s="82" t="s">
+      <c r="O10" s="72" t="s">
         <v>126</v>
       </c>
       <c r="P10" s="38">
@@ -3085,96 +3232,96 @@
       <c r="R10" s="37"/>
       <c r="S10" s="58"/>
     </row>
-    <row r="11" spans="1:19" s="76" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="70"/>
-      <c r="B11" s="71">
+    <row r="11" spans="1:19" s="66" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="60"/>
+      <c r="B11" s="61">
         <f t="shared" ref="B11:B24" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
-      <c r="C11" s="72" t="s">
+      <c r="C11" s="62" t="s">
         <v>9</v>
       </c>
-      <c r="D11" s="73" t="s">
+      <c r="D11" s="63" t="s">
         <v>21</v>
       </c>
-      <c r="E11" s="73" t="s">
+      <c r="E11" s="63" t="s">
         <v>36</v>
       </c>
-      <c r="F11" s="73" t="s">
+      <c r="F11" s="63" t="s">
         <v>52</v>
       </c>
-      <c r="G11" s="73" t="s">
+      <c r="G11" s="63" t="s">
         <v>65</v>
       </c>
-      <c r="H11" s="73" t="s">
+      <c r="H11" s="63" t="s">
         <v>78</v>
       </c>
-      <c r="I11" s="73" t="s">
-        <v>127</v>
-      </c>
-      <c r="J11" s="73" t="s">
+      <c r="I11" s="63" t="s">
+        <v>127</v>
+      </c>
+      <c r="J11" s="63" t="s">
         <v>90</v>
       </c>
-      <c r="K11" s="73" t="s">
+      <c r="K11" s="63" t="s">
         <v>104</v>
       </c>
-      <c r="L11" s="73">
+      <c r="L11" s="63">
         <v>1</v>
       </c>
       <c r="M11" s="37">
-        <f t="shared" ref="M11:M25" si="1">L11*10</f>
+        <f t="shared" ref="M11:M27" si="1">L11*10</f>
         <v>10</v>
       </c>
-      <c r="N11" s="73">
+      <c r="N11" s="63">
         <v>20</v>
       </c>
-      <c r="O11" s="84" t="s">
+      <c r="O11" s="74" t="s">
         <v>126</v>
       </c>
-      <c r="P11" s="74">
+      <c r="P11" s="64">
         <v>2.3300000000000001E-2</v>
       </c>
-      <c r="Q11" s="74">
+      <c r="Q11" s="64">
         <f t="shared" ref="Q11" si="2">P11*N11</f>
         <v>0.46600000000000003</v>
       </c>
-      <c r="R11" s="73"/>
-      <c r="S11" s="73"/>
-    </row>
-    <row r="12" spans="1:19" s="76" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="70"/>
-      <c r="B12" s="77">
+      <c r="R11" s="63"/>
+      <c r="S11" s="63"/>
+    </row>
+    <row r="12" spans="1:19" s="66" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="60"/>
+      <c r="B12" s="67">
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
-      <c r="C12" s="72" t="s">
+      <c r="C12" s="62" t="s">
         <v>9</v>
       </c>
-      <c r="D12" s="79" t="s">
+      <c r="D12" s="69" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="79" t="s">
+      <c r="E12" s="69" t="s">
         <v>37</v>
       </c>
-      <c r="F12" s="79" t="s">
+      <c r="F12" s="69" t="s">
         <v>53</v>
       </c>
-      <c r="G12" s="79" t="s">
+      <c r="G12" s="69" t="s">
         <v>66</v>
       </c>
-      <c r="H12" s="79" t="s">
+      <c r="H12" s="69" t="s">
         <v>77</v>
       </c>
-      <c r="I12" s="79" t="s">
-        <v>127</v>
-      </c>
-      <c r="J12" s="79" t="s">
+      <c r="I12" s="69" t="s">
+        <v>127</v>
+      </c>
+      <c r="J12" s="69" t="s">
         <v>91</v>
       </c>
-      <c r="K12" s="79" t="s">
+      <c r="K12" s="69" t="s">
         <v>105</v>
       </c>
-      <c r="L12" s="79">
+      <c r="L12" s="69">
         <v>2</v>
       </c>
       <c r="M12" s="37">
@@ -3184,165 +3331,165 @@
       <c r="N12" s="37">
         <v>40</v>
       </c>
-      <c r="O12" s="82" t="s">
+      <c r="O12" s="72" t="s">
         <v>126</v>
       </c>
       <c r="P12" s="38">
         <v>3.5200000000000002E-2</v>
       </c>
-      <c r="Q12" s="80">
+      <c r="Q12" s="70">
         <f>P12*N12</f>
         <v>1.4080000000000001</v>
       </c>
-      <c r="R12" s="79"/>
-      <c r="S12" s="75"/>
-    </row>
-    <row r="13" spans="1:19" s="76" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="70"/>
-      <c r="B13" s="77">
+      <c r="R12" s="69"/>
+      <c r="S12" s="65"/>
+    </row>
+    <row r="13" spans="1:19" s="66" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="60"/>
+      <c r="B13" s="67">
         <f>ROW(B13) - ROW($B$9)</f>
         <v>4</v>
       </c>
-      <c r="C13" s="72" t="s">
+      <c r="C13" s="62" t="s">
         <v>9</v>
       </c>
-      <c r="D13" s="79" t="s">
+      <c r="D13" s="69" t="s">
         <v>23</v>
       </c>
-      <c r="E13" s="79" t="s">
+      <c r="E13" s="69" t="s">
         <v>38</v>
       </c>
-      <c r="F13" s="79" t="s">
+      <c r="F13" s="69" t="s">
         <v>52</v>
       </c>
-      <c r="G13" s="79" t="s">
+      <c r="G13" s="69" t="s">
         <v>67</v>
       </c>
-      <c r="H13" s="79" t="s">
+      <c r="H13" s="69" t="s">
         <v>79</v>
       </c>
-      <c r="I13" s="79" t="s">
-        <v>127</v>
-      </c>
-      <c r="J13" s="79" t="s">
+      <c r="I13" s="69" t="s">
+        <v>127</v>
+      </c>
+      <c r="J13" s="69" t="s">
         <v>92</v>
       </c>
-      <c r="K13" s="79" t="s">
+      <c r="K13" s="69" t="s">
         <v>107</v>
       </c>
-      <c r="L13" s="79">
+      <c r="L13" s="69">
         <v>4</v>
       </c>
       <c r="M13" s="37">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="N13" s="79">
+      <c r="N13" s="69">
         <v>50</v>
       </c>
-      <c r="O13" s="83" t="s">
+      <c r="O13" s="73" t="s">
         <v>126</v>
       </c>
-      <c r="P13" s="80">
+      <c r="P13" s="70">
         <v>1.0800000000000001E-2</v>
       </c>
-      <c r="Q13" s="80">
+      <c r="Q13" s="70">
         <f>P13*N13</f>
         <v>0.54</v>
       </c>
-      <c r="R13" s="79"/>
-      <c r="S13" s="75"/>
-    </row>
-    <row r="14" spans="1:19" s="76" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="70"/>
-      <c r="B14" s="71">
+      <c r="R13" s="69"/>
+      <c r="S13" s="65"/>
+    </row>
+    <row r="14" spans="1:19" s="66" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="60"/>
+      <c r="B14" s="61">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="72" t="s">
+      <c r="C14" s="62" t="s">
         <v>9</v>
       </c>
-      <c r="D14" s="73" t="s">
+      <c r="D14" s="63" t="s">
         <v>24</v>
       </c>
-      <c r="E14" s="73" t="s">
+      <c r="E14" s="63" t="s">
         <v>39</v>
       </c>
-      <c r="F14" s="73" t="s">
+      <c r="F14" s="63" t="s">
         <v>52</v>
       </c>
-      <c r="G14" s="73" t="s">
+      <c r="G14" s="63" t="s">
         <v>68</v>
       </c>
-      <c r="H14" s="73" t="s">
+      <c r="H14" s="63" t="s">
         <v>77</v>
       </c>
-      <c r="I14" s="73" t="s">
-        <v>127</v>
-      </c>
-      <c r="J14" s="73" t="s">
+      <c r="I14" s="63" t="s">
+        <v>127</v>
+      </c>
+      <c r="J14" s="63" t="s">
         <v>93</v>
       </c>
-      <c r="K14" s="73" t="s">
+      <c r="K14" s="63" t="s">
         <v>108</v>
       </c>
-      <c r="L14" s="73">
+      <c r="L14" s="63">
         <v>1</v>
       </c>
       <c r="M14" s="37">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N14" s="73">
+      <c r="N14" s="63">
         <v>100</v>
       </c>
-      <c r="O14" s="84" t="s">
+      <c r="O14" s="74" t="s">
         <v>126</v>
       </c>
-      <c r="P14" s="74">
+      <c r="P14" s="64">
         <v>1.1000000000000001E-3</v>
       </c>
-      <c r="Q14" s="74">
+      <c r="Q14" s="64">
         <f t="shared" ref="Q14" si="3">P14*N14</f>
         <v>0.11</v>
       </c>
-      <c r="R14" s="73"/>
-      <c r="S14" s="75"/>
-    </row>
-    <row r="15" spans="1:19" s="76" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A15" s="70"/>
-      <c r="B15" s="71">
+      <c r="R14" s="63"/>
+      <c r="S14" s="65"/>
+    </row>
+    <row r="15" spans="1:19" s="66" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A15" s="60"/>
+      <c r="B15" s="61">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="72" t="s">
+      <c r="C15" s="62" t="s">
         <v>9</v>
       </c>
       <c r="D15" s="49" t="s">
         <v>128</v>
       </c>
-      <c r="E15" s="73" t="s">
+      <c r="E15" s="63" t="s">
         <v>40</v>
       </c>
-      <c r="F15" s="73" t="s">
+      <c r="F15" s="63" t="s">
         <v>52</v>
       </c>
-      <c r="G15" s="73" t="s">
+      <c r="G15" s="63" t="s">
         <v>69</v>
       </c>
-      <c r="H15" s="73" t="s">
+      <c r="H15" s="63" t="s">
         <v>77</v>
       </c>
-      <c r="I15" s="73" t="s">
-        <v>127</v>
-      </c>
-      <c r="J15" s="73" t="s">
+      <c r="I15" s="63" t="s">
+        <v>127</v>
+      </c>
+      <c r="J15" s="63" t="s">
         <v>94</v>
       </c>
-      <c r="K15" s="73" t="s">
+      <c r="K15" s="63" t="s">
         <v>106</v>
       </c>
-      <c r="L15" s="73">
+      <c r="L15" s="63">
         <v>11</v>
       </c>
       <c r="M15" s="37">
@@ -3352,53 +3499,53 @@
       <c r="N15" s="37">
         <v>200</v>
       </c>
-      <c r="O15" s="82" t="s">
+      <c r="O15" s="72" t="s">
         <v>126</v>
       </c>
       <c r="P15" s="38">
         <v>1.1000000000000001E-3</v>
       </c>
-      <c r="Q15" s="74">
+      <c r="Q15" s="64">
         <f t="shared" ref="Q15" si="4">P15*N15</f>
         <v>0.22</v>
       </c>
-      <c r="R15" s="73"/>
-      <c r="S15" s="75"/>
-    </row>
-    <row r="16" spans="1:19" s="76" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="70"/>
-      <c r="B16" s="77">
+      <c r="R15" s="63"/>
+      <c r="S15" s="65"/>
+    </row>
+    <row r="16" spans="1:19" s="66" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="60"/>
+      <c r="B16" s="67">
         <f>ROW(B16) - ROW($B$9)</f>
         <v>7</v>
       </c>
-      <c r="C16" s="78" t="s">
+      <c r="C16" s="68" t="s">
         <v>10</v>
       </c>
-      <c r="D16" s="79" t="s">
+      <c r="D16" s="69" t="s">
         <v>25</v>
       </c>
-      <c r="E16" s="79" t="s">
+      <c r="E16" s="69" t="s">
         <v>41</v>
       </c>
-      <c r="F16" s="79" t="s">
+      <c r="F16" s="69" t="s">
         <v>54</v>
       </c>
-      <c r="G16" s="79" t="s">
+      <c r="G16" s="69" t="s">
         <v>70</v>
       </c>
-      <c r="H16" s="79" t="s">
+      <c r="H16" s="69" t="s">
         <v>80</v>
       </c>
-      <c r="I16" s="79" t="s">
-        <v>127</v>
-      </c>
-      <c r="J16" s="79" t="s">
+      <c r="I16" s="69" t="s">
+        <v>127</v>
+      </c>
+      <c r="J16" s="69" t="s">
         <v>95</v>
       </c>
-      <c r="K16" s="79" t="s">
+      <c r="K16" s="69" t="s">
         <v>109</v>
       </c>
-      <c r="L16" s="79">
+      <c r="L16" s="69">
         <v>7</v>
       </c>
       <c r="M16" s="37">
@@ -3408,53 +3555,53 @@
       <c r="N16" s="37">
         <v>100</v>
       </c>
-      <c r="O16" s="82" t="s">
+      <c r="O16" s="72" t="s">
         <v>126</v>
       </c>
       <c r="P16" s="38">
         <v>5.5999999999999999E-3</v>
       </c>
-      <c r="Q16" s="80">
+      <c r="Q16" s="70">
         <f>P16*N16</f>
         <v>0.55999999999999994</v>
       </c>
-      <c r="R16" s="79"/>
-      <c r="S16" s="75"/>
-    </row>
-    <row r="17" spans="1:19" s="76" customFormat="1" ht="48" x14ac:dyDescent="0.25">
-      <c r="A17" s="70"/>
-      <c r="B17" s="71">
+      <c r="R16" s="69"/>
+      <c r="S16" s="65"/>
+    </row>
+    <row r="17" spans="1:19" s="66" customFormat="1" ht="48" x14ac:dyDescent="0.25">
+      <c r="A17" s="60"/>
+      <c r="B17" s="61">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="72" t="s">
+      <c r="C17" s="62" t="s">
         <v>11</v>
       </c>
-      <c r="D17" s="73" t="s">
+      <c r="D17" s="63" t="s">
         <v>26</v>
       </c>
       <c r="E17" s="49" t="s">
         <v>42</v>
       </c>
-      <c r="F17" s="73" t="s">
+      <c r="F17" s="63" t="s">
         <v>125</v>
       </c>
-      <c r="G17" s="73" t="s">
+      <c r="G17" s="63" t="s">
         <v>55</v>
       </c>
-      <c r="H17" s="73" t="s">
+      <c r="H17" s="63" t="s">
         <v>81</v>
       </c>
-      <c r="I17" s="73" t="s">
-        <v>127</v>
-      </c>
-      <c r="J17" s="73" t="s">
+      <c r="I17" s="63" t="s">
+        <v>127</v>
+      </c>
+      <c r="J17" s="63" t="s">
         <v>96</v>
       </c>
-      <c r="K17" s="73" t="s">
-        <v>127</v>
-      </c>
-      <c r="L17" s="73">
+      <c r="K17" s="63" t="s">
+        <v>127</v>
+      </c>
+      <c r="L17" s="63">
         <v>1</v>
       </c>
       <c r="M17" s="37">
@@ -3464,74 +3611,74 @@
       <c r="N17" s="49">
         <v>15</v>
       </c>
-      <c r="O17" s="82" t="s">
+      <c r="O17" s="72" t="s">
         <v>126</v>
       </c>
       <c r="P17" s="50">
         <v>8.6599999999999996E-2</v>
       </c>
-      <c r="Q17" s="74">
+      <c r="Q17" s="64">
         <f t="shared" ref="Q17" si="5">P17*N17</f>
         <v>1.2989999999999999</v>
       </c>
-      <c r="R17" s="73"/>
-      <c r="S17" s="75"/>
-    </row>
-    <row r="18" spans="1:19" s="76" customFormat="1" ht="24" x14ac:dyDescent="0.25">
-      <c r="A18" s="70"/>
-      <c r="B18" s="77">
+      <c r="R17" s="63"/>
+      <c r="S17" s="65"/>
+    </row>
+    <row r="18" spans="1:19" s="66" customFormat="1" ht="24" x14ac:dyDescent="0.25">
+      <c r="A18" s="60"/>
+      <c r="B18" s="67">
         <f>ROW(B18) - ROW($B$9)</f>
         <v>9</v>
       </c>
-      <c r="C18" s="78" t="s">
+      <c r="C18" s="68" t="s">
         <v>12</v>
       </c>
-      <c r="D18" s="79" t="s">
+      <c r="D18" s="69" t="s">
         <v>27</v>
       </c>
       <c r="E18" s="37" t="s">
         <v>43</v>
       </c>
-      <c r="F18" s="79" t="s">
+      <c r="F18" s="69" t="s">
         <v>125</v>
       </c>
-      <c r="G18" s="79" t="s">
+      <c r="G18" s="69" t="s">
         <v>56</v>
       </c>
-      <c r="H18" s="79" t="s">
+      <c r="H18" s="69" t="s">
         <v>82</v>
       </c>
-      <c r="I18" s="79" t="s">
-        <v>127</v>
-      </c>
-      <c r="J18" s="79" t="s">
+      <c r="I18" s="69" t="s">
+        <v>127</v>
+      </c>
+      <c r="J18" s="69" t="s">
         <v>97</v>
       </c>
-      <c r="K18" s="79" t="s">
-        <v>127</v>
-      </c>
-      <c r="L18" s="79">
+      <c r="K18" s="69" t="s">
+        <v>127</v>
+      </c>
+      <c r="L18" s="69">
         <v>5</v>
       </c>
       <c r="M18" s="37">
         <f t="shared" si="1"/>
         <v>50</v>
       </c>
-      <c r="N18" s="79">
+      <c r="N18" s="69">
         <v>55</v>
       </c>
-      <c r="O18" s="83" t="s">
+      <c r="O18" s="73" t="s">
         <v>126</v>
       </c>
-      <c r="P18" s="80">
+      <c r="P18" s="70">
         <v>0.16700000000000001</v>
       </c>
-      <c r="Q18" s="80">
+      <c r="Q18" s="70">
         <f>P18*N18</f>
         <v>9.1850000000000005</v>
       </c>
-      <c r="R18" s="79"/>
-      <c r="S18" s="75"/>
+      <c r="R18" s="69"/>
+      <c r="S18" s="65"/>
     </row>
     <row r="19" spans="1:19" s="59" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="57"/>
@@ -3542,437 +3689,549 @@
       <c r="C19" s="51" t="s">
         <v>13</v>
       </c>
-      <c r="D19" s="85" t="s">
+      <c r="D19" s="75" t="s">
         <v>28</v>
       </c>
-      <c r="E19" s="85" t="s">
+      <c r="E19" s="75" t="s">
         <v>44</v>
       </c>
-      <c r="F19" s="85" t="s">
-        <v>127</v>
-      </c>
-      <c r="G19" s="85" t="s">
+      <c r="F19" s="75" t="s">
+        <v>127</v>
+      </c>
+      <c r="G19" s="75" t="s">
         <v>57</v>
       </c>
-      <c r="H19" s="85" t="s">
-        <v>127</v>
-      </c>
-      <c r="I19" s="85" t="s">
-        <v>127</v>
-      </c>
-      <c r="J19" s="85" t="s">
-        <v>127</v>
-      </c>
-      <c r="K19" s="85" t="s">
-        <v>127</v>
-      </c>
-      <c r="L19" s="85">
+      <c r="H19" s="75" t="s">
+        <v>127</v>
+      </c>
+      <c r="I19" s="75" t="s">
+        <v>127</v>
+      </c>
+      <c r="J19" s="75" t="s">
+        <v>127</v>
+      </c>
+      <c r="K19" s="75" t="s">
+        <v>127</v>
+      </c>
+      <c r="L19" s="75">
         <v>1</v>
       </c>
-      <c r="M19" s="85">
+      <c r="M19" s="75">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N19" s="85" t="s">
-        <v>127</v>
-      </c>
-      <c r="O19" s="85" t="s">
-        <v>127</v>
-      </c>
-      <c r="P19" s="86" t="s">
-        <v>127</v>
-      </c>
-      <c r="Q19" s="86" t="s">
-        <v>127</v>
-      </c>
-      <c r="R19" s="85"/>
-      <c r="S19" s="87"/>
-    </row>
-    <row r="20" spans="1:19" s="76" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="70"/>
-      <c r="B20" s="71">
+      <c r="N19" s="75" t="s">
+        <v>127</v>
+      </c>
+      <c r="O19" s="75" t="s">
+        <v>127</v>
+      </c>
+      <c r="P19" s="76" t="s">
+        <v>127</v>
+      </c>
+      <c r="Q19" s="76" t="s">
+        <v>127</v>
+      </c>
+      <c r="R19" s="75"/>
+      <c r="S19" s="77"/>
+    </row>
+    <row r="20" spans="1:19" s="66" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="60"/>
+      <c r="B20" s="61">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C20" s="72" t="s">
+      <c r="C20" s="62" t="s">
         <v>14</v>
       </c>
-      <c r="D20" s="73" t="s">
+      <c r="D20" s="63" t="s">
         <v>29</v>
       </c>
-      <c r="E20" s="73" t="s">
+      <c r="E20" s="63" t="s">
         <v>45</v>
       </c>
-      <c r="F20" s="73" t="s">
+      <c r="F20" s="63" t="s">
         <v>58</v>
       </c>
-      <c r="G20" s="73" t="s">
+      <c r="G20" s="63" t="s">
         <v>71</v>
       </c>
-      <c r="H20" s="73" t="s">
+      <c r="H20" s="63" t="s">
         <v>83</v>
       </c>
-      <c r="I20" s="73"/>
-      <c r="J20" s="73" t="s">
+      <c r="I20" s="63"/>
+      <c r="J20" s="63" t="s">
         <v>98</v>
       </c>
-      <c r="K20" s="73" t="s">
+      <c r="K20" s="63" t="s">
         <v>111</v>
       </c>
-      <c r="L20" s="73">
+      <c r="L20" s="63">
         <v>1</v>
       </c>
       <c r="M20" s="37">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N20" s="73">
+      <c r="N20" s="63">
         <v>50</v>
       </c>
-      <c r="O20" s="84" t="s">
+      <c r="O20" s="74" t="s">
         <v>126</v>
       </c>
-      <c r="P20" s="74">
+      <c r="P20" s="64">
         <v>3.5999999999999999E-3</v>
       </c>
-      <c r="Q20" s="74">
+      <c r="Q20" s="64">
         <f t="shared" ref="Q20" si="6">P20*N20</f>
         <v>0.18</v>
       </c>
-      <c r="R20" s="73"/>
-      <c r="S20" s="75"/>
-    </row>
-    <row r="21" spans="1:19" s="76" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="70"/>
-      <c r="B21" s="77">
+      <c r="R20" s="63"/>
+      <c r="S20" s="65"/>
+    </row>
+    <row r="21" spans="1:19" s="66" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="60"/>
+      <c r="B21" s="67">
         <f>ROW(B21) - ROW($B$9)</f>
         <v>12</v>
       </c>
-      <c r="C21" s="78" t="s">
+      <c r="C21" s="68" t="s">
         <v>14</v>
       </c>
-      <c r="D21" s="79" t="s">
+      <c r="D21" s="69" t="s">
         <v>129</v>
       </c>
-      <c r="E21" s="79" t="s">
+      <c r="E21" s="69" t="s">
         <v>46</v>
       </c>
-      <c r="F21" s="79" t="s">
+      <c r="F21" s="69" t="s">
         <v>59</v>
       </c>
-      <c r="G21" s="79" t="s">
+      <c r="G21" s="69" t="s">
         <v>72</v>
       </c>
-      <c r="H21" s="79" t="s">
+      <c r="H21" s="69" t="s">
         <v>77</v>
       </c>
-      <c r="I21" s="79" t="s">
-        <v>127</v>
-      </c>
-      <c r="J21" s="79" t="s">
+      <c r="I21" s="69" t="s">
+        <v>127</v>
+      </c>
+      <c r="J21" s="69" t="s">
         <v>99</v>
       </c>
-      <c r="K21" s="79" t="s">
+      <c r="K21" s="69" t="s">
         <v>110</v>
       </c>
-      <c r="L21" s="79">
-        <v>4</v>
+      <c r="L21" s="69">
+        <v>5</v>
       </c>
       <c r="M21" s="37">
         <f t="shared" si="1"/>
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="N21" s="49">
         <v>100</v>
       </c>
-      <c r="O21" s="82" t="s">
+      <c r="O21" s="72" t="s">
         <v>126</v>
       </c>
       <c r="P21" s="50">
         <v>1E-3</v>
       </c>
-      <c r="Q21" s="80">
+      <c r="Q21" s="70">
         <f>P21*N21</f>
         <v>0.1</v>
       </c>
-      <c r="R21" s="79"/>
-      <c r="S21" s="75"/>
-    </row>
-    <row r="22" spans="1:19" s="76" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="70"/>
-      <c r="B22" s="71">
+      <c r="R21" s="69"/>
+      <c r="S21" s="65"/>
+    </row>
+    <row r="22" spans="1:19" s="66" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="60"/>
+      <c r="B22" s="61">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C22" s="72" t="s">
+      <c r="C22" s="62" t="s">
         <v>15</v>
       </c>
-      <c r="D22" s="73" t="s">
+      <c r="D22" s="63" t="s">
         <v>30</v>
       </c>
-      <c r="E22" s="73" t="s">
+      <c r="E22" s="63" t="s">
         <v>47</v>
       </c>
-      <c r="F22" s="73" t="s">
+      <c r="F22" s="63" t="s">
         <v>60</v>
       </c>
-      <c r="G22" s="73" t="s">
+      <c r="G22" s="63" t="s">
         <v>73</v>
       </c>
-      <c r="H22" s="73" t="s">
+      <c r="H22" s="63" t="s">
         <v>84</v>
       </c>
-      <c r="I22" s="73" t="s">
-        <v>127</v>
-      </c>
-      <c r="J22" s="73"/>
-      <c r="K22" s="73" t="s">
-        <v>127</v>
-      </c>
-      <c r="L22" s="73">
+      <c r="I22" s="63" t="s">
+        <v>127</v>
+      </c>
+      <c r="J22" s="63"/>
+      <c r="K22" s="63" t="s">
+        <v>127</v>
+      </c>
+      <c r="L22" s="63">
         <v>1</v>
       </c>
       <c r="M22" s="37">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N22" s="73"/>
-      <c r="O22" s="73"/>
-      <c r="P22" s="74"/>
-      <c r="Q22" s="74">
+      <c r="N22" s="63"/>
+      <c r="O22" s="63"/>
+      <c r="P22" s="64"/>
+      <c r="Q22" s="64">
         <f t="shared" ref="Q22" si="7">P22*N22</f>
         <v>0</v>
       </c>
-      <c r="R22" s="73"/>
-      <c r="S22" s="75"/>
-    </row>
-    <row r="23" spans="1:19" s="76" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="70"/>
-      <c r="B23" s="77">
+      <c r="R22" s="63"/>
+      <c r="S22" s="65"/>
+    </row>
+    <row r="23" spans="1:19" s="66" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="60"/>
+      <c r="B23" s="67">
         <f>ROW(B23) - ROW($B$9)</f>
         <v>14</v>
       </c>
-      <c r="C23" s="78" t="s">
+      <c r="C23" s="68" t="s">
         <v>16</v>
       </c>
-      <c r="D23" s="79" t="s">
+      <c r="D23" s="69" t="s">
         <v>31</v>
       </c>
-      <c r="E23" s="79" t="s">
+      <c r="E23" s="69" t="s">
         <v>48</v>
       </c>
-      <c r="F23" s="79" t="s">
+      <c r="F23" s="69" t="s">
         <v>61</v>
       </c>
-      <c r="G23" s="79" t="s">
+      <c r="G23" s="69" t="s">
         <v>74</v>
       </c>
-      <c r="H23" s="79" t="s">
+      <c r="H23" s="69" t="s">
         <v>85</v>
       </c>
-      <c r="I23" s="79" t="s">
-        <v>127</v>
-      </c>
-      <c r="J23" s="79" t="s">
+      <c r="I23" s="69" t="s">
+        <v>127</v>
+      </c>
+      <c r="J23" s="69" t="s">
         <v>100</v>
       </c>
-      <c r="K23" s="79" t="s">
-        <v>127</v>
-      </c>
-      <c r="L23" s="79">
+      <c r="K23" s="69" t="s">
+        <v>127</v>
+      </c>
+      <c r="L23" s="69">
         <v>1</v>
       </c>
       <c r="M23" s="37">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N23" s="79">
+      <c r="N23" s="69">
         <v>11</v>
       </c>
-      <c r="O23" s="83" t="s">
+      <c r="O23" s="73" t="s">
         <v>126</v>
       </c>
-      <c r="P23" s="80">
+      <c r="P23" s="70">
         <v>0.31190000000000001</v>
       </c>
-      <c r="Q23" s="80">
+      <c r="Q23" s="70">
         <f>P23*N23</f>
         <v>3.4309000000000003</v>
       </c>
-      <c r="R23" s="79"/>
-      <c r="S23" s="75"/>
-    </row>
-    <row r="24" spans="1:19" s="76" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="70"/>
-      <c r="B24" s="71">
+      <c r="R23" s="69"/>
+      <c r="S23" s="65"/>
+    </row>
+    <row r="24" spans="1:19" s="66" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="60"/>
+      <c r="B24" s="61">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C24" s="72" t="s">
+      <c r="C24" s="62" t="s">
         <v>17</v>
       </c>
-      <c r="D24" s="73" t="s">
+      <c r="D24" s="63" t="s">
         <v>32</v>
       </c>
-      <c r="E24" s="73" t="s">
+      <c r="E24" s="63" t="s">
         <v>49</v>
       </c>
-      <c r="F24" s="73" t="s">
+      <c r="F24" s="63" t="s">
         <v>125</v>
       </c>
-      <c r="G24" s="73" t="s">
+      <c r="G24" s="63" t="s">
         <v>62</v>
       </c>
-      <c r="H24" s="73" t="s">
+      <c r="H24" s="63" t="s">
         <v>86</v>
       </c>
-      <c r="I24" s="73" t="s">
-        <v>127</v>
-      </c>
-      <c r="J24" s="73" t="s">
+      <c r="I24" s="63" t="s">
+        <v>127</v>
+      </c>
+      <c r="J24" s="63" t="s">
         <v>101</v>
       </c>
-      <c r="K24" s="73" t="s">
-        <v>127</v>
-      </c>
-      <c r="L24" s="73">
+      <c r="K24" s="63" t="s">
+        <v>127</v>
+      </c>
+      <c r="L24" s="63">
         <v>4</v>
       </c>
       <c r="M24" s="37">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="N24" s="73">
+      <c r="N24" s="63">
         <v>41</v>
       </c>
-      <c r="O24" s="84" t="s">
+      <c r="O24" s="74" t="s">
         <v>126</v>
       </c>
-      <c r="P24" s="74">
+      <c r="P24" s="64">
         <v>1.7676000000000001</v>
       </c>
-      <c r="Q24" s="74">
+      <c r="Q24" s="64">
         <f t="shared" ref="Q24" si="8">P24*N24</f>
         <v>72.471600000000009</v>
       </c>
-      <c r="R24" s="73"/>
-      <c r="S24" s="75"/>
-    </row>
-    <row r="25" spans="1:19" s="76" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="70"/>
-      <c r="B25" s="77">
+      <c r="R24" s="63"/>
+      <c r="S24" s="65"/>
+    </row>
+    <row r="25" spans="1:19" s="66" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="60"/>
+      <c r="B25" s="67">
         <f>ROW(B25) - ROW($B$9)</f>
         <v>16</v>
       </c>
-      <c r="C25" s="78" t="s">
+      <c r="C25" s="68" t="s">
         <v>18</v>
       </c>
-      <c r="D25" s="79" t="s">
+      <c r="D25" s="69" t="s">
         <v>33</v>
       </c>
-      <c r="E25" s="79" t="s">
+      <c r="E25" s="69" t="s">
         <v>50</v>
       </c>
-      <c r="F25" s="79" t="s">
+      <c r="F25" s="69" t="s">
         <v>125</v>
       </c>
-      <c r="G25" s="79" t="s">
+      <c r="G25" s="69" t="s">
         <v>75</v>
       </c>
-      <c r="H25" s="79" t="s">
+      <c r="H25" s="69" t="s">
         <v>87</v>
       </c>
-      <c r="I25" s="79" t="s">
-        <v>127</v>
-      </c>
-      <c r="J25" s="79" t="s">
+      <c r="I25" s="69" t="s">
+        <v>127</v>
+      </c>
+      <c r="J25" s="69" t="s">
         <v>102</v>
       </c>
-      <c r="K25" s="79" t="s">
+      <c r="K25" s="69" t="s">
         <v>112</v>
       </c>
-      <c r="L25" s="79">
+      <c r="L25" s="69">
         <v>1</v>
       </c>
       <c r="M25" s="37">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N25" s="79">
+      <c r="N25" s="69">
         <v>11</v>
       </c>
-      <c r="O25" s="83" t="s">
+      <c r="O25" s="73" t="s">
         <v>126</v>
       </c>
-      <c r="P25" s="80">
+      <c r="P25" s="70">
         <v>0.86070000000000002</v>
       </c>
-      <c r="Q25" s="80">
+      <c r="Q25" s="70">
         <f>P25*N25</f>
         <v>9.4677000000000007</v>
       </c>
-      <c r="R25" s="79"/>
-      <c r="S25" s="81"/>
-    </row>
-    <row r="26" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R25" s="69"/>
+      <c r="S25" s="71"/>
+    </row>
+    <row r="26" spans="1:19" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
-      <c r="B26" s="39"/>
-      <c r="C26" s="40"/>
-      <c r="D26" s="41"/>
-      <c r="E26" s="42"/>
-      <c r="F26" s="43"/>
-      <c r="G26" s="44"/>
-      <c r="H26" s="43"/>
-      <c r="I26" s="44"/>
-      <c r="J26" s="43"/>
-      <c r="K26" s="44"/>
-      <c r="L26" s="44"/>
-      <c r="M26" s="44"/>
-      <c r="N26" s="68" t="s">
+      <c r="B26" s="67">
+        <f t="shared" ref="B26:B27" si="9">ROW(B26) - ROW($B$9)</f>
+        <v>17</v>
+      </c>
+      <c r="C26" s="68" t="s">
+        <v>134</v>
+      </c>
+      <c r="D26" s="69" t="s">
+        <v>141</v>
+      </c>
+      <c r="E26" s="37" t="s">
+        <v>136</v>
+      </c>
+      <c r="F26" s="69" t="s">
+        <v>127</v>
+      </c>
+      <c r="G26" s="37" t="s">
+        <v>135</v>
+      </c>
+      <c r="H26" s="69" t="s">
+        <v>137</v>
+      </c>
+      <c r="I26" s="63" t="s">
+        <v>127</v>
+      </c>
+      <c r="J26" s="69" t="s">
+        <v>138</v>
+      </c>
+      <c r="K26" s="69" t="s">
+        <v>127</v>
+      </c>
+      <c r="L26" s="69">
+        <v>1</v>
+      </c>
+      <c r="M26" s="37">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="N26" s="69">
+        <v>11</v>
+      </c>
+      <c r="O26" s="73" t="s">
+        <v>126</v>
+      </c>
+      <c r="P26" s="70">
+        <v>0.17219999999999999</v>
+      </c>
+      <c r="Q26" s="70">
+        <f>P26*N26</f>
+        <v>1.8941999999999999</v>
+      </c>
+      <c r="R26" s="69"/>
+      <c r="S26" s="71"/>
+    </row>
+    <row r="27" spans="1:19" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="1"/>
+      <c r="B27" s="67">
+        <f t="shared" si="9"/>
+        <v>18</v>
+      </c>
+      <c r="C27" s="68" t="s">
+        <v>134</v>
+      </c>
+      <c r="D27" s="69" t="s">
+        <v>142</v>
+      </c>
+      <c r="E27" s="37" t="s">
+        <v>140</v>
+      </c>
+      <c r="F27" s="69" t="s">
+        <v>127</v>
+      </c>
+      <c r="G27" s="69" t="s">
+        <v>139</v>
+      </c>
+      <c r="H27" s="69" t="s">
+        <v>143</v>
+      </c>
+      <c r="I27" s="69" t="s">
+        <v>127</v>
+      </c>
+      <c r="J27" s="69" t="s">
+        <v>144</v>
+      </c>
+      <c r="K27" s="69" t="s">
+        <v>127</v>
+      </c>
+      <c r="L27" s="69">
+        <v>1</v>
+      </c>
+      <c r="M27" s="37">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="N27" s="69">
+        <v>15</v>
+      </c>
+      <c r="O27" s="73" t="s">
+        <v>126</v>
+      </c>
+      <c r="P27" s="70">
+        <v>8.0600000000000005E-2</v>
+      </c>
+      <c r="Q27" s="70">
+        <f>P27*N27</f>
+        <v>1.2090000000000001</v>
+      </c>
+      <c r="R27" s="69"/>
+      <c r="S27" s="71"/>
+    </row>
+    <row r="28" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="1"/>
+      <c r="B28" s="39"/>
+      <c r="C28" s="40"/>
+      <c r="D28" s="41"/>
+      <c r="E28" s="42"/>
+      <c r="F28" s="43"/>
+      <c r="G28" s="44"/>
+      <c r="H28" s="43"/>
+      <c r="I28" s="44"/>
+      <c r="J28" s="43"/>
+      <c r="K28" s="44"/>
+      <c r="L28" s="44"/>
+      <c r="M28" s="44"/>
+      <c r="N28" s="82" t="s">
         <v>5</v>
       </c>
-      <c r="O26" s="69"/>
-      <c r="P26" s="69"/>
-      <c r="Q26" s="47">
+      <c r="O28" s="83"/>
+      <c r="P28" s="83"/>
+      <c r="Q28" s="47">
         <f>SUM(Q10:Q25)</f>
         <v>99.918200000000013</v>
       </c>
-      <c r="R26" s="64"/>
-      <c r="S26" s="65"/>
-    </row>
-    <row r="27" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="1"/>
-      <c r="B27" s="25"/>
-      <c r="C27" s="36"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="10"/>
-      <c r="F27" s="10"/>
-      <c r="G27" s="10"/>
-      <c r="H27" s="10"/>
-      <c r="I27" s="10"/>
-      <c r="J27" s="10"/>
-      <c r="K27" s="10"/>
-      <c r="L27" s="10"/>
-      <c r="M27" s="10"/>
-      <c r="N27" s="68" t="s">
+      <c r="R28" s="84"/>
+      <c r="S28" s="85"/>
+    </row>
+    <row r="29" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="1"/>
+      <c r="B29" s="25"/>
+      <c r="C29" s="36"/>
+      <c r="D29" s="9"/>
+      <c r="E29" s="10"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="10"/>
+      <c r="H29" s="10"/>
+      <c r="I29" s="10"/>
+      <c r="J29" s="10"/>
+      <c r="K29" s="10"/>
+      <c r="L29" s="10"/>
+      <c r="M29" s="10"/>
+      <c r="N29" s="82" t="s">
         <v>6</v>
       </c>
-      <c r="O27" s="69"/>
-      <c r="P27" s="69"/>
-      <c r="Q27" s="48">
-        <f>Q26/10</f>
+      <c r="O29" s="83"/>
+      <c r="P29" s="83"/>
+      <c r="Q29" s="48">
+        <f>Q28/10</f>
         <v>9.9918200000000006</v>
       </c>
-      <c r="R27" s="66"/>
-      <c r="S27" s="67"/>
+      <c r="R29" s="86"/>
+      <c r="S29" s="87"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="K1:S1"/>
     <mergeCell ref="S3:S8"/>
-    <mergeCell ref="N26:P26"/>
-    <mergeCell ref="R26:S27"/>
-    <mergeCell ref="N27:P27"/>
+    <mergeCell ref="N28:P28"/>
+    <mergeCell ref="R28:S29"/>
+    <mergeCell ref="N29:P29"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="O10" r:id="rId1"/>
@@ -3989,9 +4248,11 @@
     <hyperlink ref="O13" r:id="rId12"/>
     <hyperlink ref="O14" r:id="rId13"/>
     <hyperlink ref="O20" r:id="rId14"/>
+    <hyperlink ref="O26" r:id="rId15"/>
+    <hyperlink ref="O27" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId15"/>
-  <drawing r:id="rId16"/>
+  <pageSetup orientation="portrait" r:id="rId17"/>
+  <drawing r:id="rId18"/>
 </worksheet>
 </file>
</xml_diff>